<commit_message>
Take the automatic colors of Excel charts from the workbook's theme
A series (or pie slice) without a color of its own gets the color Excel
would give it: from the chart's color style (colorsN.xml, "Change
Colors") or else the theme's accent1-6, repeated with the default
variations. Luminance modifiers are applied in HSL as Office does, which
also makes theme colors with lumMod/lumOff match Excel exactly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014LqK3aNKHwEJScab7Lf8qd
</commit_message>
<xml_diff>
--- a/testdata/xlsx/charts.xlsx
+++ b/testdata/xlsx/charts.xlsx
@@ -1383,6 +1383,17 @@
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="15">
+  <a:schemeClr val="accent6"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+</cs:colorStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>